<commit_message>
Start populating with v7 data
</commit_message>
<xml_diff>
--- a/Raw_Data/12.xlsx
+++ b/Raw_Data/12.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://anthesisllc-my.sharepoint.com/personal/lovisa_areback_anthesisgroup_com/Documents/Dokument/GitHub/CBA_GBG_PROT/Input/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\StefanÅström\C_Verktyg\Python\ALL_PYTHON\2026_v7_Goth_Prot_CBA\Raw_Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="16" documentId="8_{6875EADB-AFAD-4E79-A326-5762FBACA071}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{73DFF123-C9AF-4D06-A9D2-5EFAC63F3170}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1F01C458-E395-47CF-AA68-C93D4CCE630C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-23550" yWindow="135" windowWidth="21930" windowHeight="12975" activeTab="2" xr2:uid="{0EFAC0D5-3333-49E4-993E-3033691A9986}"/>
+    <workbookView xWindow="28680" yWindow="-2850" windowWidth="38640" windowHeight="21120" xr2:uid="{0EFAC0D5-3333-49E4-993E-3033691A9986}"/>
   </bookViews>
   <sheets>
     <sheet name="INFO" sheetId="49" r:id="rId1"/>
@@ -1240,15 +1240,15 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>1</xdr:col>
-      <xdr:colOff>9526</xdr:colOff>
+      <xdr:colOff>11431</xdr:colOff>
       <xdr:row>3</xdr:row>
-      <xdr:rowOff>171450</xdr:rowOff>
+      <xdr:rowOff>167639</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>12</xdr:col>
-      <xdr:colOff>561976</xdr:colOff>
-      <xdr:row>60</xdr:row>
-      <xdr:rowOff>85726</xdr:rowOff>
+      <xdr:colOff>560071</xdr:colOff>
+      <xdr:row>63</xdr:row>
+      <xdr:rowOff>47624</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
@@ -1263,8 +1263,8 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="619126" y="742950"/>
-          <a:ext cx="7524750" cy="10772776"/>
+          <a:off x="621031" y="710564"/>
+          <a:ext cx="7559040" cy="10738485"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -3145,14 +3145,14 @@
     <tabColor rgb="FF90E1FA"/>
   </sheetPr>
   <dimension ref="B2:R22"/>
-  <sheetFormatPr defaultRowHeight="14.6"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="2" max="2" width="10.69140625" customWidth="1"/>
-    <col min="3" max="3" width="11.53515625" customWidth="1"/>
-    <col min="15" max="15" width="34.4609375" customWidth="1"/>
-    <col min="16" max="16" width="16.3046875" customWidth="1"/>
-    <col min="17" max="17" width="22.3046875" customWidth="1"/>
-    <col min="18" max="18" width="17.07421875" customWidth="1"/>
+    <col min="2" max="2" width="10.6640625" customWidth="1"/>
+    <col min="3" max="3" width="11.5546875" customWidth="1"/>
+    <col min="15" max="15" width="34.44140625" customWidth="1"/>
+    <col min="16" max="16" width="16.33203125" customWidth="1"/>
+    <col min="17" max="17" width="22.33203125" customWidth="1"/>
+    <col min="18" max="18" width="17.109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="2:18">
@@ -3427,17 +3427,17 @@
     <tabColor rgb="FFCCFFCC"/>
   </sheetPr>
   <dimension ref="A1:I953"/>
-  <sheetFormatPr defaultColWidth="9.07421875" defaultRowHeight="14.6"/>
+  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="22.4609375" style="16" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="25.53515625" style="63" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="22.23046875" style="15" customWidth="1"/>
-    <col min="4" max="4" width="24.07421875" style="17" customWidth="1"/>
+    <col min="1" max="1" width="22.44140625" style="16" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="25.5546875" style="63" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="22.21875" style="15" customWidth="1"/>
+    <col min="4" max="4" width="24.109375" style="17" customWidth="1"/>
     <col min="5" max="5" width="19" style="42" customWidth="1"/>
-    <col min="6" max="6" width="9.07421875" style="1"/>
-    <col min="7" max="7" width="17.07421875" style="1" customWidth="1"/>
-    <col min="8" max="8" width="7.53515625" style="1" customWidth="1"/>
-    <col min="9" max="16384" width="9.07421875" style="1"/>
+    <col min="6" max="6" width="9.109375" style="1"/>
+    <col min="7" max="7" width="17.109375" style="1" customWidth="1"/>
+    <col min="8" max="8" width="7.5546875" style="1" customWidth="1"/>
+    <col min="9" max="16384" width="9.109375" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9" s="4" customFormat="1" ht="15" thickBot="1">
@@ -19672,13 +19672,13 @@
     <tabColor rgb="FFCCFFCC"/>
   </sheetPr>
   <dimension ref="A1:E57"/>
-  <sheetFormatPr defaultColWidth="9.07421875" defaultRowHeight="14.6"/>
+  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="22.4609375" style="14" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="9.07421875" style="27"/>
-    <col min="3" max="3" width="11.4609375" style="28" customWidth="1"/>
-    <col min="4" max="4" width="9.07421875" style="29"/>
-    <col min="5" max="16384" width="9.07421875" style="1"/>
+    <col min="1" max="1" width="22.44140625" style="14" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.109375" style="27"/>
+    <col min="3" max="3" width="11.44140625" style="28" customWidth="1"/>
+    <col min="4" max="4" width="9.109375" style="29"/>
+    <col min="5" max="16384" width="9.109375" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" s="10" customFormat="1" ht="15" thickBot="1">
@@ -20489,19 +20489,19 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9B7D634B-8F05-4D0E-8573-40905363F18A}">
   <dimension ref="A1:H50"/>
-  <sheetFormatPr defaultRowHeight="14.6"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="24" customWidth="1"/>
-    <col min="2" max="2" width="51.4609375" customWidth="1"/>
-    <col min="3" max="3" width="10.4609375" style="59" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="19.53515625" style="59" customWidth="1"/>
-    <col min="5" max="5" width="12.07421875" style="59" customWidth="1"/>
-    <col min="6" max="6" width="21.3046875" style="59" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="30.69140625" style="59" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="51.44140625" customWidth="1"/>
+    <col min="3" max="3" width="10.44140625" style="59" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="19.5546875" style="59" customWidth="1"/>
+    <col min="5" max="5" width="12.109375" style="59" customWidth="1"/>
+    <col min="6" max="6" width="21.33203125" style="59" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="30.6640625" style="59" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="11" style="59" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" s="47" customFormat="1" ht="14.15">
+    <row r="1" spans="1:8" s="47" customFormat="1" ht="13.8">
       <c r="A1" s="43" t="s">
         <v>112</v>
       </c>
@@ -20853,7 +20853,7 @@
       <c r="G21" s="50"/>
       <c r="H21" s="51"/>
     </row>
-    <row r="22" spans="1:8" ht="18.899999999999999">
+    <row r="22" spans="1:8" ht="18.600000000000001">
       <c r="A22" s="48" t="s">
         <v>89</v>
       </c>
@@ -21332,6 +21332,17 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="bdc51464-d60a-4b5b-8137-84cff6a8af51">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="caf619d2-c8b4-4eae-8df0-1f9a9957400a" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="dokument" ma:contentTypeID="0x0101002EF99EFDC33C6E41B104484FD3E0D8C6" ma:contentTypeVersion="17" ma:contentTypeDescription="Skapa ett nytt dokument." ma:contentTypeScope="" ma:versionID="22c1f030af46f95256dc74e55c4240ba">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="bdc51464-d60a-4b5b-8137-84cff6a8af51" xmlns:ns3="caf619d2-c8b4-4eae-8df0-1f9a9957400a" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="9ad56c7555e4f778ea2176d4266d1773" ns2:_="" ns3:_="">
     <xsd:import namespace="bdc51464-d60a-4b5b-8137-84cff6a8af51"/>
@@ -21580,17 +21591,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="bdc51464-d60a-4b5b-8137-84cff6a8af51">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="caf619d2-c8b4-4eae-8df0-1f9a9957400a" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{345157FC-9AB7-471E-8A38-484235567C74}">
   <ds:schemaRefs>
@@ -21600,6 +21600,17 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FA28B098-AA57-4494-8DA3-761B84790965}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="bdc51464-d60a-4b5b-8137-84cff6a8af51"/>
+    <ds:schemaRef ds:uri="caf619d2-c8b4-4eae-8df0-1f9a9957400a"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{82159ACA-EC17-4838-94D2-64960F74C798}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -21616,15 +21627,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FA28B098-AA57-4494-8DA3-761B84790965}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="bdc51464-d60a-4b5b-8137-84cff6a8af51"/>
-    <ds:schemaRef ds:uri="caf619d2-c8b4-4eae-8df0-1f9a9957400a"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>